<commit_message>
Ask for fewer default-app changes, fix a Quick Look crash on close
macOS 26.4 and later make the user confirm every file type an app
wants to open by default. Make Default now covers the five that matter
most (PDF, Word, CSV, Markdown, plain text) and changes them one at a
time; older Word formats, TSV, JSON, logs, code and images are a
checkbox away in Settings, or make-default --all.

Also:
- A Quick Look preview closed before it started loading no longer
  takes the app down.
- The smoke test prints crash reports, and on macOS 26 records what
  macOS shows when asked to change the default app.
- A fuller spreadsheet sample for the Quick Look screenshot.
</commit_message>
<xml_diff>
--- a/Samples/Budget.xlsx
+++ b/Samples/Budget.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suppliers" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,19 +29,40 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Helvetica Neue"/>
+      <color rgb="0026222F"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Helvetica Neue"/>
       <b val="1"/>
       <color rgb="0026222F"/>
-      <sz val="14"/>
+      <sz val="16"/>
     </font>
     <font>
+      <name val="Helvetica Neue"/>
+      <color rgb="007A7185"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Helvetica Neue"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="12"/>
     </font>
     <font>
+      <name val="Helvetica Neue"/>
       <b val="1"/>
+      <color rgb="0026222F"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Helvetica Neue"/>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -52,8 +74,13 @@
         <fgColor rgb="00F86F5B"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDF3EC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -62,23 +89,53 @@
       <diagonal/>
     </border>
     <border>
+      <bottom style="thin">
+        <color rgb="00EADFD6"/>
+      </bottom>
+    </border>
+    <border>
       <top style="medium">
         <color rgb="0026222F"/>
       </top>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -444,200 +501,547 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Harbor Street Bakery — Q4 budget</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+          <t>Harbor Street Bakery — second half budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>July to December 2026 · all three shops</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>October</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>November</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>December</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Aug</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Dec</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="5" ht="19" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Flour &amp; grain</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B5" s="6" t="n">
+        <v>4100</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>4150</v>
+      </c>
+      <c r="D5" s="6" t="n">
         <v>4200</v>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="E5" s="6" t="n">
+        <v>4200</v>
+      </c>
+      <c r="F5" s="6" t="n">
         <v>4300</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="G5" s="6" t="n">
         <v>4900</v>
       </c>
-      <c r="E4" s="3" t="n">
-        <v>13400</v>
+      <c r="H5" s="7" t="n">
+        <v>25850</v>
+      </c>
+    </row>
+    <row r="6" ht="19" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Butter &amp; dairy</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>3050</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>3100</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>3100</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>3150</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>3600</v>
+      </c>
+      <c r="H6" s="10" t="n">
+        <v>19000</v>
+      </c>
+    </row>
+    <row r="7" ht="19" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Eggs</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>900</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>920</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>940</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>950</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>980</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>1150</v>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>5840</v>
+      </c>
+    </row>
+    <row r="8" ht="19" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Coffee beans</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>1750</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>1800</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>1780</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>1750</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>2100</v>
+      </c>
+      <c r="H8" s="10" t="n">
+        <v>10980</v>
+      </c>
+    </row>
+    <row r="9" ht="19" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Fruit &amp; nuts</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>1200</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>1350</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>1100</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>1050</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>7400</v>
+      </c>
+    </row>
+    <row r="10" ht="19" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Wages</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>21000</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>21200</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>21300</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>21500</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>21500</v>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>24800</v>
+      </c>
+      <c r="H10" s="10" t="n">
+        <v>131300</v>
+      </c>
+    </row>
+    <row r="11" ht="19" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Rent</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>6200</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>6200</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>6200</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>6200</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>6200</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>6200</v>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>37200</v>
+      </c>
+    </row>
+    <row r="12" ht="19" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>1350</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>1300</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>1400</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>1450</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>1900</v>
+      </c>
+      <c r="H12" s="10" t="n">
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="13" ht="19" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Packaging</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>600</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>610</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>615</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>620</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>640</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>900</v>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>3985</v>
+      </c>
+    </row>
+    <row r="14" ht="19" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Repairs</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="n">
+        <v>250</v>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>480</v>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>120</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>300</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>1150</v>
+      </c>
+    </row>
+    <row r="15" ht="19" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="n">
+        <v>40350</v>
+      </c>
+      <c r="C15" s="12" t="n">
+        <v>40580</v>
+      </c>
+      <c r="D15" s="12" t="n">
+        <v>41315</v>
+      </c>
+      <c r="E15" s="12" t="n">
+        <v>40920</v>
+      </c>
+      <c r="F15" s="12" t="n">
+        <v>41290</v>
+      </c>
+      <c r="G15" s="12" t="n">
+        <v>47250</v>
+      </c>
+      <c r="H15" s="12" t="n">
+        <v>251705</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Suppliers</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Who we order from, and when</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Supplies</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Order day</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Terms</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Butter &amp; dairy</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>3100</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>3150</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>3600</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>9850</v>
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Millbrook Flour</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Flour, rye, spelt</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>30 days</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>Green Valley Dairy</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Butter, milk, cream</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>Mon &amp; Thu</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>14 days</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>Harbor Roasters</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Coffee beans</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
-        <v>1800</v>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>1750</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>2100</v>
-      </c>
-      <c r="E6" s="3" t="n">
-        <v>5650</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Wages</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n">
-        <v>21500</v>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>21500</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>24800</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>67800</v>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>30 days</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Rent</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="n">
-        <v>6200</v>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>6200</v>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>6200</v>
-      </c>
-      <c r="E8" s="3" t="n">
-        <v>18600</v>
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Orchard Lane</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Fruit, nuts</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>On delivery</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>1450</v>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>1600</v>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>1900</v>
-      </c>
-      <c r="E9" s="3" t="n">
-        <v>4950</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Packaging</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>620</v>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>640</v>
-      </c>
-      <c r="D10" s="3" t="n">
-        <v>900</v>
-      </c>
-      <c r="E10" s="3" t="n">
-        <v>2160</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="n">
-        <v>38870</v>
-      </c>
-      <c r="C11" s="5" t="n">
-        <v>39140</v>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>44400</v>
-      </c>
-      <c r="E11" s="5" t="n">
-        <v>122410</v>
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>Paper &amp; Co</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Boxes, bags, cups</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>30 days</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Size Settings to each pane, tidy the Word and Excel samples
- The Settings window now resizes to fit whichever pane is showing.
  Before, the AI pane was cut off below the review rules.
- The Word sample's table has borders Quick Look can draw, and the
  spreadsheet's title no longer runs under gridlines.
- macOS only asks when Handa takes a file type over from another app,
  so the messages say it may ask rather than that it will.
</commit_message>
<xml_diff>
--- a/Samples/Budget.xlsx
+++ b/Samples/Budget.xlsx
@@ -879,6 +879,10 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1045,6 +1049,10 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>